<commit_message>
improvement on HeroX fuel raising and droping
</commit_message>
<xml_diff>
--- a/data/mym/Libro1.xlsx
+++ b/data/mym/Libro1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose.Hurtado\Documents\Zonar_projects\data\mym\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED09805-7D43-445B-80FE-DB07FC881722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB185A3B-BCEC-44CD-8A6D-DE211A91A996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4EB0C79B-B897-4039-93C6-82940471E36A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
   <si>
     <t>ncode</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>litros</t>
+  </si>
+  <si>
+    <t>Cambio</t>
   </si>
 </sst>
 </file>
@@ -169,7 +172,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,6 +182,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -195,11 +204,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -228,7 +239,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>885494</xdr:colOff>
+      <xdr:colOff>740714</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>99767</xdr:rowOff>
     </xdr:to>
@@ -265,13 +276,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>762000</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>137160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
+      <xdr:col>22</xdr:col>
       <xdr:colOff>609600</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
@@ -644,7 +655,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B7485B-D7BD-4DC1-8E5F-CA0E69016F79}">
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
@@ -652,16 +663,17 @@
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.109375" customWidth="1"/>
-    <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="14.109375" customWidth="1"/>
+    <col min="9" max="9" width="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -680,24 +692,28 @@
       <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="1"/>
-      <c r="I1">
+      <c r="G1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="1"/>
+      <c r="J1">
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="J1">
+      <c r="K1">
         <v>4.7161</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2640</v>
       </c>
@@ -712,22 +728,22 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>2798</v>
       </c>
-      <c r="K2">
-        <f>H2*I$1-J$1</f>
+      <c r="L2">
+        <f>I2*J$1-K$1</f>
         <v>179.95189999999999</v>
       </c>
-      <c r="L2">
-        <f>K2/3.7854</f>
+      <c r="M2">
+        <f>L2/3.7854</f>
         <v>47.538410735985629</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2656</v>
       </c>
@@ -742,22 +758,30 @@
       <c r="F3" t="s">
         <v>5</v>
       </c>
-      <c r="H3">
+      <c r="G3">
+        <f>E3-E2</f>
+        <v>0.43662492735245451</v>
+      </c>
+      <c r="I3">
         <v>2903</v>
       </c>
-      <c r="K3">
-        <f t="shared" ref="K3:K17" si="2">H3*I$1-J$1</f>
+      <c r="L3">
+        <f t="shared" ref="L3:L17" si="2">I3*J$1-K$1</f>
         <v>186.8819</v>
       </c>
-      <c r="L3">
-        <f t="shared" ref="L3:L17" si="3">K3/3.7854</f>
+      <c r="M3">
+        <f t="shared" ref="M3:M17" si="3">L3/3.7854</f>
         <v>49.369128757859144</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O3">
+        <f>M3-M2</f>
+        <v>1.8307180218735155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2991</v>
       </c>
@@ -772,22 +796,30 @@
       <c r="F4" t="s">
         <v>7</v>
       </c>
-      <c r="H4">
+      <c r="G4">
+        <f t="shared" ref="G4:G18" si="4">E4-E3</f>
+        <v>9.1418344164421228</v>
+      </c>
+      <c r="I4">
         <v>4095</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O4">
+        <f t="shared" ref="O4:O17" si="5">M4-M3</f>
+        <v>20.783008400697426</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3869</v>
       </c>
@@ -802,23 +834,31 @@
       <c r="F5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="1"/>
-      <c r="H5">
+      <c r="G5">
+        <f t="shared" si="4"/>
+        <v>23.959792888466225</v>
+      </c>
+      <c r="H5" s="1"/>
+      <c r="I5">
         <v>4095</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O5">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4000</v>
       </c>
@@ -833,23 +873,31 @@
       <c r="F6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="1"/>
-      <c r="H6">
+      <c r="G6">
+        <f t="shared" si="4"/>
+        <v>3.5748665926982426</v>
+      </c>
+      <c r="H6" s="1"/>
+      <c r="I6">
         <v>4095</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O6">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>4016</v>
       </c>
@@ -864,28 +912,36 @@
       <c r="F7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="1"/>
-      <c r="H7">
+      <c r="G7">
+        <f t="shared" si="4"/>
+        <v>0.43662492735246872</v>
+      </c>
+      <c r="H7" s="1"/>
+      <c r="I7">
         <v>4095</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O7">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>4009</v>
       </c>
       <c r="D8">
-        <f t="shared" ref="D8:D17" si="4">A8*B$1-C$1</f>
+        <f t="shared" ref="D8:D18" si="6">A8*B$1-C$1</f>
         <v>409.86450000000002</v>
       </c>
       <c r="E8">
@@ -895,28 +951,36 @@
       <c r="F8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="1"/>
-      <c r="H8">
+      <c r="G8">
+        <f t="shared" si="4"/>
+        <v>-0.19102340571669174</v>
+      </c>
+      <c r="H8" s="1"/>
+      <c r="I8">
         <v>4095</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M8" t="s">
+      <c r="N8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O8">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>4020</v>
       </c>
       <c r="D9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>411.00080000000003</v>
       </c>
       <c r="E9">
@@ -926,28 +990,36 @@
       <c r="F9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="1"/>
-      <c r="H9">
+      <c r="G9">
+        <f t="shared" si="4"/>
+        <v>0.30017963755480537</v>
+      </c>
+      <c r="H9" s="1"/>
+      <c r="I9">
         <v>4095</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L9">
+      <c r="M9">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M9" t="s">
+      <c r="N9" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O9">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>4034</v>
       </c>
       <c r="D10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>412.447</v>
       </c>
       <c r="E10">
@@ -957,29 +1029,37 @@
       <c r="F10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="1"/>
-      <c r="H10">
+      <c r="G10">
+        <f t="shared" si="4"/>
+        <v>0.38204681143339769</v>
+      </c>
+      <c r="H10" s="1"/>
+      <c r="I10">
         <v>4095</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L10">
+      <c r="M10">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M10" t="s">
+      <c r="N10" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O10">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>4045</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>413.58330000000001</v>
       </c>
       <c r="E11">
@@ -989,29 +1069,37 @@
       <c r="F11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="1"/>
-      <c r="H11">
+      <c r="G11">
+        <f t="shared" si="4"/>
+        <v>0.30017963755481958</v>
+      </c>
+      <c r="H11" s="1"/>
+      <c r="I11">
         <v>4095</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M11" t="s">
+      <c r="N11" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O11">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>4048</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>413.89320000000004</v>
       </c>
       <c r="E12">
@@ -1021,29 +1109,37 @@
       <c r="F12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="1"/>
-      <c r="H12">
+      <c r="G12">
+        <f t="shared" si="4"/>
+        <v>8.1867173878592325E-2</v>
+      </c>
+      <c r="H12" s="1"/>
+      <c r="I12">
         <v>4095</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L12">
+      <c r="M12">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M12" t="s">
+      <c r="N12" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O12">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>4055</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>414.61630000000002</v>
       </c>
       <c r="E13">
@@ -1053,29 +1149,37 @@
       <c r="F13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G13" s="1"/>
-      <c r="H13">
+      <c r="G13">
+        <f t="shared" si="4"/>
+        <v>0.19102340571670595</v>
+      </c>
+      <c r="H13" s="1"/>
+      <c r="I13">
         <v>4095</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L13">
+      <c r="M13">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M13" t="s">
+      <c r="N13" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O13">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>4071</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>416.26910000000004</v>
       </c>
       <c r="E14">
@@ -1085,29 +1189,37 @@
       <c r="F14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G14" s="1"/>
-      <c r="H14">
+      <c r="G14">
+        <f t="shared" si="4"/>
+        <v>0.43662492735245451</v>
+      </c>
+      <c r="H14" s="1"/>
+      <c r="I14">
         <v>4095</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L14">
+      <c r="M14">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M14" t="s">
+      <c r="N14" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O14">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>4057</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>414.8229</v>
       </c>
       <c r="E15">
@@ -1117,29 +1229,37 @@
       <c r="F15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G15" s="1"/>
-      <c r="H15">
+      <c r="G15">
+        <f t="shared" si="4"/>
+        <v>-0.3820468114334119</v>
+      </c>
+      <c r="H15" s="1"/>
+      <c r="I15">
         <v>4095</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L15">
+      <c r="M15">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M15" t="s">
+      <c r="N15" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O15">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>4063</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>415.4427</v>
       </c>
       <c r="E16">
@@ -1149,109 +1269,154 @@
       <c r="F16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G16" s="1"/>
-      <c r="H16">
+      <c r="G16">
+        <f t="shared" si="4"/>
+        <v>0.16373434775717044</v>
+      </c>
+      <c r="H16" s="1"/>
+      <c r="I16">
         <v>4095</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L16">
+      <c r="M16">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M16" t="s">
+      <c r="N16" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>4087</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>417.92189999999999</v>
       </c>
       <c r="E17">
-        <f t="shared" si="1"/>
+        <f>D17/3.7854</f>
         <v>110.40362973529878</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G17" s="1"/>
-      <c r="H17">
+      <c r="G17">
+        <f t="shared" si="4"/>
+        <v>0.65493739102869597</v>
+      </c>
+      <c r="H17" s="1"/>
+      <c r="I17">
         <v>4095</v>
       </c>
-      <c r="K17">
+      <c r="L17">
         <f t="shared" si="2"/>
         <v>265.55390000000006</v>
       </c>
-      <c r="L17">
+      <c r="M17">
         <f t="shared" si="3"/>
         <v>70.15213715855657</v>
       </c>
-      <c r="M17" t="s">
+      <c r="N17" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="C18" s="2"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O17">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A18" s="4">
+        <v>4046</v>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="4">
+        <f t="shared" si="6"/>
+        <v>413.6866</v>
+      </c>
+      <c r="E18" s="4">
+        <f>D18/3.7854</f>
+        <v>109.28477835895809</v>
+      </c>
+      <c r="F18" s="4"/>
+      <c r="G18">
+        <f t="shared" si="4"/>
+        <v>-1.118851376340686</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C19" s="2"/>
       <c r="E19" s="3">
         <f>E17-E2</f>
         <v>39.487266867438052</v>
       </c>
-      <c r="L19" s="3">
-        <f>L17-L2</f>
+      <c r="G19" s="4">
+        <f>SUM(G3:G18)</f>
+        <v>38.368415491097366</v>
+      </c>
+      <c r="M19" s="3">
+        <f>M17-M2</f>
         <v>22.613726422570942</v>
       </c>
-      <c r="M19" s="3">
-        <f>E19+L19</f>
+      <c r="N19" s="3">
+        <f>E19+M19</f>
         <v>62.100993290008994</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O19" s="4">
+        <f>SUM(O3:O17)</f>
+        <v>22.613726422570942</v>
+      </c>
+      <c r="P19" s="4">
+        <f>G19+O19</f>
+        <v>60.982141913668308</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C20" s="2"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C21" s="2"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C22" s="2"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C23" s="2"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C24" s="2"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C25" s="2"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C26" s="2"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C27" s="2"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C28" s="2"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C29" s="2"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C30" s="2"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C31" s="2"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C32" s="2"/>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.3">

</xml_diff>